<commit_message>
Reset workbook opening positions to first visible worksheet
Save the current workbook revisions and ensure all 22 workbooks open at A1 on their first visible worksheet. Preserve workbook contents while updating the saved view settings.
</commit_message>
<xml_diff>
--- a/ch_02/ch_02_solution.xlsx
+++ b/ch_02/ch_02_solution.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30515"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30610"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GeorgeMount\Documents\GitHub\Python-in-Excel-for-Data-Analytics\ch_02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57BAB798-30DC-45AB-BE45-757F4853DD5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5150410-B72E-4E57-98AD-204ECFE28472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="18915" windowHeight="12676" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="18915" windowHeight="12676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nyc" sheetId="1" r:id="rId1"/>
@@ -6717,132 +6717,132 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A18">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="B18" t="str">
-        <v>ORD-0111</v>
+        <v>ORD-0041</v>
       </c>
       <c r="C18" t="str">
-        <v>Keyboard</v>
+        <v>Bookshelf</v>
       </c>
       <c r="D18" t="str">
-        <v>Electronics</v>
+        <v>Furniture</v>
       </c>
       <c r="E18">
-        <v>475.83</v>
+        <v>751.03</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G18">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="H18" t="str">
-        <v>United States</v>
+        <v>Germany</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A19">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="B19" t="str">
-        <v>ORD-0163</v>
+        <v>ORD-0177</v>
       </c>
       <c r="C19" t="str">
-        <v>Binder</v>
+        <v>Printer Paper</v>
       </c>
       <c r="D19" t="str">
         <v>Office Supplies</v>
       </c>
       <c r="E19">
-        <v>33.159999999999997</v>
+        <v>25.53</v>
       </c>
       <c r="F19">
-        <v>2</v>
-      </c>
-      <c r="G19" t="e">
-        <v>#NUM!</v>
+        <v>8</v>
+      </c>
+      <c r="G19">
+        <v>26</v>
       </c>
       <c r="H19" t="str">
-        <v>United States</v>
+        <v>Canada</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A20">
+        <v>55</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ORD-0056</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Printer Paper</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Office Supplies</v>
+      </c>
+      <c r="E20">
+        <v>43.21</v>
+      </c>
+      <c r="F20">
         <v>4</v>
       </c>
-      <c r="B20" t="str">
-        <v>ORD-0005</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Tablet</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Electronics</v>
-      </c>
-      <c r="E20">
-        <v>479.68</v>
-      </c>
-      <c r="F20">
-        <v>6</v>
-      </c>
       <c r="G20">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H20" t="str">
-        <v>United States</v>
+        <v>Canada</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A21">
-        <v>102</v>
+        <v>157</v>
       </c>
       <c r="B21" t="str">
-        <v>ORD-0103</v>
+        <v>ORD-0158</v>
       </c>
       <c r="C21" t="str">
-        <v>Bookshelf</v>
+        <v>Headphones</v>
       </c>
       <c r="D21" t="str">
-        <v>Furniture</v>
+        <v>Electronics</v>
       </c>
       <c r="E21">
-        <v>369.13</v>
+        <v>459.17</v>
       </c>
       <c r="F21">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G21">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H21" t="str">
-        <v>United States</v>
+        <v>Germany</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A22">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="B22" t="str">
-        <v>ORD-0161</v>
+        <v>ORD-0170</v>
       </c>
       <c r="C22" t="str">
-        <v>Binder</v>
+        <v>Keyboard</v>
       </c>
       <c r="D22" t="str">
-        <v>Office Supplies</v>
+        <v>Electronics</v>
       </c>
       <c r="E22">
-        <v>30.06</v>
+        <v>122.47</v>
       </c>
       <c r="F22">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G22">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="H22" t="str">
-        <v>Germany</v>
+        <v>United Kingdom</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.45">
@@ -6913,7 +6913,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" t="str">
-        <v>order_id</v>
+        <v>product</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -6921,7 +6921,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" t="str">
-        <v>product</v>
+        <v>order_id</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -7281,7 +7281,7 @@
         <v>top</v>
       </c>
       <c r="B66" t="str">
-        <v>ORD-0001</v>
+        <v>ORD-0185</v>
       </c>
       <c r="C66" t="str">
         <v>Notebook</v>

</xml_diff>